<commit_message>
added marie jane metallic series
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reyesjustin/OTPROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493A1682-C14D-3043-A050-07A42B52A6B8}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5FE4E7-29DC-4F46-B3CE-A3426F529C0D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{04C67FBF-622E-F248-949E-B4D4A4FB1588}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="54">
   <si>
     <t>sku</t>
   </si>
@@ -169,6 +169,33 @@
   </si>
   <si>
     <t>Off-White/Iron Navy</t>
+  </si>
+  <si>
+    <t>1182A708-700</t>
+  </si>
+  <si>
+    <t>MEXICO 66 TGRS</t>
+  </si>
+  <si>
+    <t>Classic Red/Cream</t>
+  </si>
+  <si>
+    <t>1182A708-020</t>
+  </si>
+  <si>
+    <t>Gunmetal/Metropilos</t>
+  </si>
+  <si>
+    <t>1182A708-250</t>
+  </si>
+  <si>
+    <t>Champagne/Cream</t>
+  </si>
+  <si>
+    <t>1182A708-701</t>
+  </si>
+  <si>
+    <t>Crystal Pink/Cream</t>
   </si>
 </sst>
 </file>
@@ -195,15 +222,16 @@
       <name val="Matter SQ , sans-serif"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF4B4F54"/>
-      <name val="Matter SQ , sans-serif"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF4B4F54"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -226,12 +254,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -546,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B21564-E78C-9647-A1D3-B4D73713D832}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.33203125" customWidth="1"/>
@@ -727,7 +754,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B11" t="s">
@@ -863,9 +890,75 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="3"/>
+      <c r="A19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added the rest of the marie jane series
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reyesjustin/OTPROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5FE4E7-29DC-4F46-B3CE-A3426F529C0D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F61587F-71B9-4344-8F79-EA40134F63C7}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{04C67FBF-622E-F248-949E-B4D4A4FB1588}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="61">
   <si>
     <t>sku</t>
   </si>
@@ -196,6 +196,27 @@
   </si>
   <si>
     <t>Crystal Pink/Cream</t>
+  </si>
+  <si>
+    <t>1182A678-700</t>
+  </si>
+  <si>
+    <t>1182A678-750</t>
+  </si>
+  <si>
+    <t>1182A678-200</t>
+  </si>
+  <si>
+    <t>1182A678-001</t>
+  </si>
+  <si>
+    <t>Crystal Pink/Graphite Grey</t>
+  </si>
+  <si>
+    <t>Birch/Peacoat</t>
+  </si>
+  <si>
+    <t>Black/Cream</t>
   </si>
 </sst>
 </file>
@@ -573,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B21564-E78C-9647-A1D3-B4D73713D832}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.33203125" customWidth="1"/>
@@ -957,6 +978,74 @@
         <v>8</v>
       </c>
     </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" t="s">
+        <v>8</v>
+      </c>
+      <c r="E24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" t="s">
+        <v>59</v>
+      </c>
+      <c r="D25" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" t="s">
+        <v>46</v>
+      </c>
+      <c r="C26" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added the full marie janes series
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reyesjustin/OTPROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F61587F-71B9-4344-8F79-EA40134F63C7}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E7FAAAF-1968-2A46-8AEE-3134D993EB0A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{04C67FBF-622E-F248-949E-B4D4A4FB1588}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="70">
   <si>
     <t>sku</t>
   </si>
@@ -217,6 +217,33 @@
   </si>
   <si>
     <t>Black/Cream</t>
+  </si>
+  <si>
+    <t>1182A705-001</t>
+  </si>
+  <si>
+    <t>1182A705-020</t>
+  </si>
+  <si>
+    <t>1182A705-250</t>
+  </si>
+  <si>
+    <t>Black/Black</t>
+  </si>
+  <si>
+    <t>Oyster Grey/Oyster Grey</t>
+  </si>
+  <si>
+    <t>Beige/Beige</t>
+  </si>
+  <si>
+    <t>1182A660-001</t>
+  </si>
+  <si>
+    <t>1182A660-752</t>
+  </si>
+  <si>
+    <t>Ivory/Cream</t>
   </si>
 </sst>
 </file>
@@ -594,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B21564-E78C-9647-A1D3-B4D73713D832}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.33203125" customWidth="1"/>
@@ -1046,6 +1073,91 @@
         <v>8</v>
       </c>
     </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" t="s">
+        <v>8</v>
+      </c>
+      <c r="E27" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" t="s">
+        <v>46</v>
+      </c>
+      <c r="C30" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" t="s">
+        <v>8</v>
+      </c>
+      <c r="E30" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" t="s">
+        <v>66</v>
+      </c>
+      <c r="D31" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added rotemit, metallic M66 SD series
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reyesjustin/OTPROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E31B5C3-578B-4C44-8903-753B1DB8E943}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7540B3-19C7-874E-860E-6AADBCDA8F85}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{04C67FBF-622E-F248-949E-B4D4A4FB1588}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="90">
   <si>
     <t>sku</t>
   </si>
@@ -244,6 +244,66 @@
   </si>
   <si>
     <t>Ivory/Cream</t>
+  </si>
+  <si>
+    <t>1183C614-750</t>
+  </si>
+  <si>
+    <t>1183C614-200</t>
+  </si>
+  <si>
+    <t>1183C614-101</t>
+  </si>
+  <si>
+    <t>1183C614-001</t>
+  </si>
+  <si>
+    <t>1183C614-100</t>
+  </si>
+  <si>
+    <t>Ivory/Oyster Grey</t>
+  </si>
+  <si>
+    <t>Birch/Deep Mars</t>
+  </si>
+  <si>
+    <t>Cream/Truffle Grey</t>
+  </si>
+  <si>
+    <t>Black/Off-White</t>
+  </si>
+  <si>
+    <t>Cream/Peacoat</t>
+  </si>
+  <si>
+    <t>1183C468-201</t>
+  </si>
+  <si>
+    <t>1183C468-400</t>
+  </si>
+  <si>
+    <t>1183C468-701</t>
+  </si>
+  <si>
+    <t>1183C468-020</t>
+  </si>
+  <si>
+    <t>1183C468-700</t>
+  </si>
+  <si>
+    <t>1183C468-200</t>
+  </si>
+  <si>
+    <t>Gold/Cream</t>
+  </si>
+  <si>
+    <t>Midnight/Cream</t>
+  </si>
+  <si>
+    <t>Metropolis/Cream</t>
+  </si>
+  <si>
+    <t>Dessert Camp/Cream</t>
   </si>
 </sst>
 </file>
@@ -621,7 +681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B21564-E78C-9647-A1D3-B4D73713D832}">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.33203125" customWidth="1"/>
@@ -1175,6 +1235,193 @@
         <v>8</v>
       </c>
     </row>
+    <row r="33" spans="1:5">
+      <c r="A33" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" t="s">
+        <v>23</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C34" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" t="s">
+        <v>8</v>
+      </c>
+      <c r="E34" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C35" t="s">
+        <v>77</v>
+      </c>
+      <c r="D35" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" t="s">
+        <v>73</v>
+      </c>
+      <c r="B36" t="s">
+        <v>23</v>
+      </c>
+      <c r="C36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" t="s">
+        <v>74</v>
+      </c>
+      <c r="B37" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" t="s">
+        <v>80</v>
+      </c>
+      <c r="B38" t="s">
+        <v>21</v>
+      </c>
+      <c r="C38" t="s">
+        <v>86</v>
+      </c>
+      <c r="D38" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" t="s">
+        <v>81</v>
+      </c>
+      <c r="B39" t="s">
+        <v>21</v>
+      </c>
+      <c r="C39" t="s">
+        <v>87</v>
+      </c>
+      <c r="D39" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" t="s">
+        <v>82</v>
+      </c>
+      <c r="B40" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" t="s">
+        <v>47</v>
+      </c>
+      <c r="D40" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" t="s">
+        <v>53</v>
+      </c>
+      <c r="D42" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" t="s">
+        <v>85</v>
+      </c>
+      <c r="B43" t="s">
+        <v>21</v>
+      </c>
+      <c r="C43" t="s">
+        <v>89</v>
+      </c>
+      <c r="D43" t="s">
+        <v>8</v>
+      </c>
+      <c r="E43" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added all the MEXICO 66 SD, excluding VIN
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reyesjustin/OTPROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7540B3-19C7-874E-860E-6AADBCDA8F85}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B1270E-6D2F-C943-8320-B882B04985F9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{04C67FBF-622E-F248-949E-B4D4A4FB1588}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="121">
   <si>
     <t>sku</t>
   </si>
@@ -304,6 +304,99 @@
   </si>
   <si>
     <t>Dessert Camp/Cream</t>
+  </si>
+  <si>
+    <t>1183A872-112</t>
+  </si>
+  <si>
+    <t>1183C345-101</t>
+  </si>
+  <si>
+    <t>11838955-020</t>
+  </si>
+  <si>
+    <t>1183C345-100</t>
+  </si>
+  <si>
+    <t>1183A592-200</t>
+  </si>
+  <si>
+    <t>1183A872-106</t>
+  </si>
+  <si>
+    <t>Cream/Pure Gold</t>
+  </si>
+  <si>
+    <t>White/Rose Gold</t>
+  </si>
+  <si>
+    <t>White/Pure Silver</t>
+  </si>
+  <si>
+    <t>Pure Silver/Cream</t>
+  </si>
+  <si>
+    <t>Birch/Silver</t>
+  </si>
+  <si>
+    <t>1183A872-101</t>
+  </si>
+  <si>
+    <t>1183A872-200</t>
+  </si>
+  <si>
+    <t>1183A872-100</t>
+  </si>
+  <si>
+    <t>1183A872-254</t>
+  </si>
+  <si>
+    <t>1183A872-003</t>
+  </si>
+  <si>
+    <t>1183A872-004</t>
+  </si>
+  <si>
+    <t>1183A872-204</t>
+  </si>
+  <si>
+    <t>1183C517-300</t>
+  </si>
+  <si>
+    <t>1183C115-001</t>
+  </si>
+  <si>
+    <t>1183C115-020</t>
+  </si>
+  <si>
+    <t>Birch/Green</t>
+  </si>
+  <si>
+    <t>Beige/Green</t>
+  </si>
+  <si>
+    <t>Black/Yellow</t>
+  </si>
+  <si>
+    <t>Licorice Brown/Champagne</t>
+  </si>
+  <si>
+    <t>Spruce Green/Mineral Beige</t>
+  </si>
+  <si>
+    <t>Metropolis/Metropolis</t>
+  </si>
+  <si>
+    <t>1183C580-020</t>
+  </si>
+  <si>
+    <t>1183C580-400</t>
+  </si>
+  <si>
+    <t>Graphite Grey/Graphite Grey</t>
+  </si>
+  <si>
+    <t>Grey Floss/Grey Floss</t>
   </si>
 </sst>
 </file>
@@ -681,7 +774,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B21564-E78C-9647-A1D3-B4D73713D832}">
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.33203125" customWidth="1"/>
@@ -1422,6 +1515,329 @@
         <v>8</v>
       </c>
     </row>
+    <row r="44" spans="1:5">
+      <c r="A44" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44" t="s">
+        <v>96</v>
+      </c>
+      <c r="D44" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" t="s">
+        <v>91</v>
+      </c>
+      <c r="B45" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" t="s">
+        <v>97</v>
+      </c>
+      <c r="D45" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" t="s">
+        <v>93</v>
+      </c>
+      <c r="B46" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46" t="s">
+        <v>98</v>
+      </c>
+      <c r="D46" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47" t="s">
+        <v>99</v>
+      </c>
+      <c r="D47" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48" t="s">
+        <v>100</v>
+      </c>
+      <c r="D48" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" t="s">
+        <v>95</v>
+      </c>
+      <c r="B49" t="s">
+        <v>21</v>
+      </c>
+      <c r="C49" t="s">
+        <v>97</v>
+      </c>
+      <c r="D49" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" t="s">
+        <v>101</v>
+      </c>
+      <c r="B50" t="s">
+        <v>21</v>
+      </c>
+      <c r="C50" t="s">
+        <v>79</v>
+      </c>
+      <c r="D50" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" t="s">
+        <v>102</v>
+      </c>
+      <c r="B51" t="s">
+        <v>21</v>
+      </c>
+      <c r="C51" t="s">
+        <v>59</v>
+      </c>
+      <c r="D51" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" t="s">
+        <v>103</v>
+      </c>
+      <c r="B52" t="s">
+        <v>21</v>
+      </c>
+      <c r="C52" t="s">
+        <v>111</v>
+      </c>
+      <c r="D52" t="s">
+        <v>8</v>
+      </c>
+      <c r="E52" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53" t="s">
+        <v>112</v>
+      </c>
+      <c r="D53" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" t="s">
+        <v>17</v>
+      </c>
+      <c r="B54" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54" t="s">
+        <v>25</v>
+      </c>
+      <c r="D54" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" t="s">
+        <v>105</v>
+      </c>
+      <c r="B55" t="s">
+        <v>21</v>
+      </c>
+      <c r="C55" t="s">
+        <v>113</v>
+      </c>
+      <c r="D55" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" t="s">
+        <v>106</v>
+      </c>
+      <c r="B56" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56" t="s">
+        <v>64</v>
+      </c>
+      <c r="D56" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
+        <v>107</v>
+      </c>
+      <c r="B57" t="s">
+        <v>21</v>
+      </c>
+      <c r="C57" t="s">
+        <v>114</v>
+      </c>
+      <c r="D57" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
+        <v>108</v>
+      </c>
+      <c r="B58" t="s">
+        <v>21</v>
+      </c>
+      <c r="C58" t="s">
+        <v>115</v>
+      </c>
+      <c r="D58" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" t="s">
+        <v>109</v>
+      </c>
+      <c r="B59" t="s">
+        <v>21</v>
+      </c>
+      <c r="C59" t="s">
+        <v>64</v>
+      </c>
+      <c r="D59" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" t="s">
+        <v>110</v>
+      </c>
+      <c r="B60" t="s">
+        <v>21</v>
+      </c>
+      <c r="C60" t="s">
+        <v>116</v>
+      </c>
+      <c r="D60" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>117</v>
+      </c>
+      <c r="B61" t="s">
+        <v>21</v>
+      </c>
+      <c r="C61" t="s">
+        <v>119</v>
+      </c>
+      <c r="D61" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" t="s">
+        <v>118</v>
+      </c>
+      <c r="B62" t="s">
+        <v>21</v>
+      </c>
+      <c r="C62" t="s">
+        <v>120</v>
+      </c>
+      <c r="D62" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added MEXICO 66 SD VIN
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reyesjustin/OTPROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B1270E-6D2F-C943-8320-B882B04985F9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F03D4B5-6CA7-0747-9670-0FA24B7A3486}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{04C67FBF-622E-F248-949E-B4D4A4FB1588}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="137">
   <si>
     <t>sku</t>
   </si>
@@ -397,6 +397,54 @@
   </si>
   <si>
     <t>Grey Floss/Grey Floss</t>
+  </si>
+  <si>
+    <t>1183C015-106</t>
+  </si>
+  <si>
+    <t>1183C015-400</t>
+  </si>
+  <si>
+    <t>1183C015-201</t>
+  </si>
+  <si>
+    <t>1183C015-104</t>
+  </si>
+  <si>
+    <t>1183C015-200</t>
+  </si>
+  <si>
+    <t>1183C015-101</t>
+  </si>
+  <si>
+    <t>Off-White/Purple Spectrum</t>
+  </si>
+  <si>
+    <t>Peacoat/Wheat Yellow</t>
+  </si>
+  <si>
+    <t>White/Director Blue</t>
+  </si>
+  <si>
+    <t>Birch/Metropolis</t>
+  </si>
+  <si>
+    <t>Cream/Birch</t>
+  </si>
+  <si>
+    <t>MEXICO 66 SD VIN</t>
+  </si>
+  <si>
+    <t>1183c105-205</t>
+  </si>
+  <si>
+    <t>1183C015-202</t>
+  </si>
+  <si>
+    <t>Beige/Beet Juice</t>
+  </si>
+  <si>
+    <t>Clay Crayon/Cream</t>
   </si>
 </sst>
 </file>
@@ -774,7 +822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B21564-E78C-9647-A1D3-B4D73713D832}">
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.33203125" customWidth="1"/>
@@ -1838,6 +1886,136 @@
         <v>8</v>
       </c>
     </row>
+    <row r="63" spans="1:5">
+      <c r="A63" t="s">
+        <v>121</v>
+      </c>
+      <c r="B63" t="s">
+        <v>132</v>
+      </c>
+      <c r="C63" t="s">
+        <v>127</v>
+      </c>
+      <c r="D63" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" t="s">
+        <v>122</v>
+      </c>
+      <c r="B64" t="s">
+        <v>132</v>
+      </c>
+      <c r="C64" t="s">
+        <v>128</v>
+      </c>
+      <c r="D64" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65" t="s">
+        <v>123</v>
+      </c>
+      <c r="B65" t="s">
+        <v>132</v>
+      </c>
+      <c r="C65" t="s">
+        <v>111</v>
+      </c>
+      <c r="D65" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" t="s">
+        <v>124</v>
+      </c>
+      <c r="B66" t="s">
+        <v>132</v>
+      </c>
+      <c r="C66" t="s">
+        <v>129</v>
+      </c>
+      <c r="D66" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" t="s">
+        <v>125</v>
+      </c>
+      <c r="B67" t="s">
+        <v>132</v>
+      </c>
+      <c r="C67" t="s">
+        <v>130</v>
+      </c>
+      <c r="D67" t="s">
+        <v>8</v>
+      </c>
+      <c r="E67" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" t="s">
+        <v>126</v>
+      </c>
+      <c r="B68" t="s">
+        <v>132</v>
+      </c>
+      <c r="C68" t="s">
+        <v>131</v>
+      </c>
+      <c r="D68" t="s">
+        <v>8</v>
+      </c>
+      <c r="E68" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" t="s">
+        <v>134</v>
+      </c>
+      <c r="C69" t="s">
+        <v>135</v>
+      </c>
+      <c r="D69" t="s">
+        <v>8</v>
+      </c>
+      <c r="E69" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" t="s">
+        <v>133</v>
+      </c>
+      <c r="C70" t="s">
+        <v>136</v>
+      </c>
+      <c r="D70" t="s">
+        <v>8</v>
+      </c>
+      <c r="E70" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixed typo on crayoncream M66 SD VIN
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reyesjustin/OTPROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3127824E-881C-D14C-A784-2070F0B31907}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2CA750-FD8B-C141-89E4-9F3A5FB07619}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{04C67FBF-622E-F248-949E-B4D4A4FB1588}"/>
   </bookViews>
@@ -435,9 +435,6 @@
     <t>MEXICO 66 SD VIN</t>
   </si>
   <si>
-    <t>1183c105-205</t>
-  </si>
-  <si>
     <t>1183C015-202</t>
   </si>
   <si>
@@ -445,6 +442,9 @@
   </si>
   <si>
     <t>Clay Crayon/Cream</t>
+  </si>
+  <si>
+    <t>1183C105-205</t>
   </si>
 </sst>
 </file>
@@ -1990,13 +1990,13 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B69" t="s">
         <v>132</v>
       </c>
       <c r="C69" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D69" t="s">
         <v>8</v>
@@ -2007,13 +2007,13 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B70" t="s">
         <v>132</v>
       </c>
       <c r="C70" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D70" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
edited product code for metallic Pure Silver/Cream
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reyesjustin/OTPROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2CA750-FD8B-C141-89E4-9F3A5FB07619}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09F6E8EB-D4FF-F343-82AC-C2D4B2F81091}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{04C67FBF-622E-F248-949E-B4D4A4FB1588}"/>
   </bookViews>
@@ -312,9 +312,6 @@
     <t>1183C345-101</t>
   </si>
   <si>
-    <t>11838955-020</t>
-  </si>
-  <si>
     <t>1183C345-100</t>
   </si>
   <si>
@@ -445,6 +442,9 @@
   </si>
   <si>
     <t>1183C105-205</t>
+  </si>
+  <si>
+    <t>1183B955-020</t>
   </si>
 </sst>
 </file>
@@ -1571,7 +1571,7 @@
         <v>21</v>
       </c>
       <c r="C44" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D44" t="s">
         <v>8</v>
@@ -1588,7 +1588,7 @@
         <v>21</v>
       </c>
       <c r="C45" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D45" t="s">
         <v>8</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B46" t="s">
         <v>21</v>
       </c>
       <c r="C46" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D46" t="s">
         <v>8</v>
@@ -1616,13 +1616,13 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>92</v>
+        <v>136</v>
       </c>
       <c r="B47" t="s">
         <v>21</v>
       </c>
       <c r="C47" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D47" t="s">
         <v>8</v>
@@ -1633,13 +1633,13 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B48" t="s">
         <v>21</v>
       </c>
       <c r="C48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D48" t="s">
         <v>8</v>
@@ -1650,13 +1650,13 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B49" t="s">
         <v>21</v>
       </c>
       <c r="C49" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D49" t="s">
         <v>8</v>
@@ -1667,7 +1667,7 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B50" t="s">
         <v>21</v>
@@ -1684,7 +1684,7 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B51" t="s">
         <v>21</v>
@@ -1701,13 +1701,13 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B52" t="s">
         <v>21</v>
       </c>
       <c r="C52" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D52" t="s">
         <v>8</v>
@@ -1718,13 +1718,13 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B53" t="s">
         <v>21</v>
       </c>
       <c r="C53" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D53" t="s">
         <v>8</v>
@@ -1752,13 +1752,13 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B55" t="s">
         <v>21</v>
       </c>
       <c r="C55" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D55" t="s">
         <v>8</v>
@@ -1769,7 +1769,7 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B56" t="s">
         <v>21</v>
@@ -1786,13 +1786,13 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B57" t="s">
         <v>21</v>
       </c>
       <c r="C57" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D57" t="s">
         <v>8</v>
@@ -1803,13 +1803,13 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B58" t="s">
         <v>21</v>
       </c>
       <c r="C58" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D58" t="s">
         <v>8</v>
@@ -1820,7 +1820,7 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B59" t="s">
         <v>21</v>
@@ -1837,13 +1837,13 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B60" t="s">
         <v>21</v>
       </c>
       <c r="C60" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D60" t="s">
         <v>8</v>
@@ -1854,13 +1854,13 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B61" t="s">
         <v>21</v>
       </c>
       <c r="C61" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D61" t="s">
         <v>8</v>
@@ -1871,13 +1871,13 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B62" t="s">
         <v>21</v>
       </c>
       <c r="C62" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D62" t="s">
         <v>8</v>
@@ -1888,13 +1888,13 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B63" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C63" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D63" t="s">
         <v>8</v>
@@ -1905,13 +1905,13 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B64" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C64" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D64" t="s">
         <v>8</v>
@@ -1922,13 +1922,13 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B65" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C65" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D65" t="s">
         <v>8</v>
@@ -1939,13 +1939,13 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B66" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C66" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D66" t="s">
         <v>8</v>
@@ -1956,13 +1956,13 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B67" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C67" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D67" t="s">
         <v>8</v>
@@ -1973,13 +1973,13 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B68" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C68" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D68" t="s">
         <v>8</v>
@@ -1990,13 +1990,13 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
+        <v>132</v>
+      </c>
+      <c r="B69" t="s">
+        <v>131</v>
+      </c>
+      <c r="C69" t="s">
         <v>133</v>
-      </c>
-      <c r="B69" t="s">
-        <v>132</v>
-      </c>
-      <c r="C69" t="s">
-        <v>134</v>
       </c>
       <c r="D69" t="s">
         <v>8</v>
@@ -2007,13 +2007,13 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B70" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C70" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D70" t="s">
         <v>8</v>

</xml_diff>